<commit_message>
Add carousel-hero, footer, header blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (14):
- .migration/plans/homepage-pixel-perfect-critique-fixes.md
- blocks/carousel-hero/carousel-hero.css
- blocks/footer/footer.css
- blocks/header/header.css
- styles/styles.css
- tools/importer/import-article.bundle.js
- tools/importer/import-article.js
- tools/importer/reports/import-article.report.xlsx
- tools/importer/reports/us/en/magazine/arctic-surfing.report.json
- tools/importer/reports/us/en/magazine/guide-la-skateparks.report.json
- tools/importer/reports/us/en/magazine/san-diego-surf.report.json
- tools/importer/reports/us/en/magazine/ski-touring.report.json
- tools/importer/reports/us/en/magazine/western-australia.report.json
- tools/importer/transformers/wknd-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="152">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-03T13:41:19.984Z</t>
+    <t>2026-09-03T18:41:53.576Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -94,7 +94,7 @@
     <t>adventures-listing</t>
   </si>
   <si>
-    <t>2026-09-03T13:41:11.744Z</t>
+    <t>2026-09-03T18:41:59.292Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -127,277 +127,280 @@
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
+    <t>["columns-featured","cards-teaser","cards-members","cards-members"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>2026-09-03T18:41:48.746Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-hero","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","tabs-detail","tabs-detail"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-09-03T11:45:24.824Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:25.488Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:32.145Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:36.580Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:41.323Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:47.446Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:29:54.464Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:00.425Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:05.023Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:10.787Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:17.248Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:22.245Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:26.883Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:32.699Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:39.083Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-03T17:30:45.609Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>us/en/magazine</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:14.245Z</t>
-  </si>
-  <si>
-    <t>Magazine</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/magazine.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp.report.json</t>
-  </si>
-  <si>
-    <t>["carousel-hero","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","columns-meta","tabs-detail","tabs-detail"]</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp</t>
-  </si>
-  <si>
-    <t>adventure-detail</t>
-  </si>
-  <si>
-    <t>2026-09-03T11:45:24.824Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:25.488Z</t>
-  </si>
-  <si>
-    <t>Beervana in Portland</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/climbing-new-zealand.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/climbing-new-zealand</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:32.145Z</t>
-  </si>
-  <si>
-    <t>Climbing New Zealand</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/colorado-rock-climbing</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:36.580Z</t>
-  </si>
-  <si>
-    <t>Colorado Rock Climbing</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/cycling-southern-utah.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/cycling-southern-utah</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:41.323Z</t>
-  </si>
-  <si>
-    <t>Cycling Southern Utah</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/cycling-tuscany.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/cycling-tuscany</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:47.446Z</t>
-  </si>
-  <si>
-    <t>Cycling Tuscany</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/downhill-skiing-wyoming</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:29:54.464Z</t>
-  </si>
-  <si>
-    <t>Downhill Skiing Wyoming</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/gastronomic-marais-tour</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:00.425Z</t>
-  </si>
-  <si>
-    <t>Gastronomic Marais Tour</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/napa-wine-tasting.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/napa-wine-tasting</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:05.023Z</t>
-  </si>
-  <si>
-    <t>Napa Wine Tasting</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/riverside-camping-australia.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/riverside-camping-australia</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:10.787Z</t>
-  </si>
-  <si>
-    <t>Riverside Camping</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/ski-touring-mont-blanc</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:17.248Z</t>
-  </si>
-  <si>
-    <t>Ski Touring Mont Blanc</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/surf-camp-costa-rica</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:22.245Z</t>
-  </si>
-  <si>
-    <t>Surf Camp in Costa Rica</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/tahoe-skiing.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/tahoe-skiing</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:26.883Z</t>
-  </si>
-  <si>
-    <t>Tahoe Skiing</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/west-coast-cycling.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/west-coast-cycling</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:32.699Z</t>
-  </si>
-  <si>
-    <t>West Coast Cycling</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/whistler-mountain-biking</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:39.083Z</t>
-  </si>
-  <si>
-    <t>Whistler Mountain Biking</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/yosemite-backpacking.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/yosemite-backpacking</t>
-  </si>
-  <si>
-    <t>2026-09-03T17:30:45.609Z</t>
-  </si>
-  <si>
-    <t>Yosemite Backpacking</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
-  </si>
-  <si>
-    <t>us/en/magazine/arctic-surfing.report.json</t>
-  </si>
-  <si>
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-03T17:16:20.403Z</t>
+    <t>2026-09-04T08:27:29.445Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -412,7 +415,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-03T17:30:57.674Z</t>
+    <t>2026-09-04T08:27:35.539Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -427,7 +430,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-03T17:31:02.724Z</t>
+    <t>2026-09-04T08:27:41.625Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -442,7 +445,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-03T17:31:09.505Z</t>
+    <t>2026-09-04T08:27:46.511Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -457,7 +460,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-03T17:31:16.631Z</t>
+    <t>2026-09-04T08:27:51.442Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -1440,129 +1443,129 @@
         <v>125</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="C24" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F25" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G25" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H25" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="C26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F26" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G27" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>